<commit_message>
Update EMOData dashboard data
</commit_message>
<xml_diff>
--- a/public/exports/11259979.xlsx
+++ b/public/exports/11259979.xlsx
@@ -281,16 +281,16 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029627</t>
+          <t xml:space="preserve">100108973</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">19</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F6">
-        <v>912</v>
+        <v>6933</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -331,16 +331,16 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">100108973</t>
+          <t xml:space="preserve">174465, 174466, 174468, 174469</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F7">
-        <v>6933</v>
+        <v>13136</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -381,16 +381,16 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">193518</t>
+          <t xml:space="preserve">174850</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="F8">
-        <v>1621</v>
+        <v>7906</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -431,16 +431,16 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">706900, 100027955</t>
+          <t xml:space="preserve">174851</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F9">
-        <v>3882</v>
+        <v>426</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -481,7 +481,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">706909, 100027932</t>
+          <t xml:space="preserve">186986, 186987, 186988, 186990</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="F10">
-        <v>892</v>
+        <v>696</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -531,30 +531,30 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029488</t>
+          <t xml:space="preserve">186989</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F11">
-        <v>7262</v>
+        <v>388</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">200060656</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">2022-07-03</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Udløbet</t>
+          <t xml:space="preserve">Mangler energimærke</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -581,7 +581,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029488</t>
+          <t xml:space="preserve">186991, 186992</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -590,21 +590,21 @@
         </is>
       </c>
       <c r="F12">
-        <v>360</v>
+        <v>428</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">200060656</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">2022-07-03</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Udløbet</t>
+          <t xml:space="preserve">Mangler energimærke</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -631,30 +631,30 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026406</t>
+          <t xml:space="preserve">187004</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F13">
-        <v>1105</v>
+        <v>586</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">311021341</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">2023-10-09</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Udløbet</t>
+          <t xml:space="preserve">Mangler energimærke</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -681,30 +681,30 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026406</t>
+          <t xml:space="preserve">187004</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F14">
-        <v>984</v>
+        <v>440</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">311021341</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t xml:space="preserve">2023-10-09</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Udløbet</t>
+          <t xml:space="preserve">Mangler energimærke</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -731,30 +731,30 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">186986, 186987, 186988, 186990</t>
+          <t xml:space="preserve">191032, 191033</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F15">
-        <v>696</v>
+        <v>1248</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">311052674</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024-05-07</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Udløbet</t>
+          <t xml:space="preserve">Mangler energimærke</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -781,30 +781,30 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">186989</t>
+          <t xml:space="preserve">191034</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F16">
-        <v>388</v>
+        <v>1225</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">311052674</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024-05-07</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Udløbet</t>
+          <t xml:space="preserve">Mangler energimærke</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">186991, 186992</t>
+          <t xml:space="preserve">193518</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -840,21 +840,21 @@
         </is>
       </c>
       <c r="F17">
-        <v>428</v>
+        <v>1621</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">311052674</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024-05-07</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Udløbet</t>
+          <t xml:space="preserve">Mangler energimærke</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -881,30 +881,30 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">706864, 100063647</t>
+          <t xml:space="preserve">706900, 100027955</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F18">
-        <v>452</v>
+        <v>3882</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">311122307</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-06-30</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Udløbet</t>
+          <t xml:space="preserve">Mangler energimærke</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025640</t>
+          <t xml:space="preserve">706909, 100027932</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -940,21 +940,21 @@
         </is>
       </c>
       <c r="F19">
-        <v>1440</v>
+        <v>892</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t xml:space="preserve">311161386</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-02-28</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Udløbet</t>
+          <t xml:space="preserve">Mangler energimærke</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025821</t>
+          <t xml:space="preserve">100026406</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -990,26 +990,26 @@
         </is>
       </c>
       <c r="F20">
-        <v>996</v>
+        <v>1105</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t xml:space="preserve">311217955</t>
+          <t xml:space="preserve">311021341</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-12-15</t>
+          <t xml:space="preserve">2023-10-09</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gyldigt</t>
+          <t xml:space="preserve">Udløbet</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nej</t>
+          <t xml:space="preserve">Ja</t>
         </is>
       </c>
     </row>
@@ -1031,35 +1031,35 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">100030255</t>
+          <t xml:space="preserve">100026406</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F21">
-        <v>413</v>
+        <v>984</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve">311218022</t>
+          <t xml:space="preserve">311021341</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-12-15</t>
+          <t xml:space="preserve">2023-10-09</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gyldigt</t>
+          <t xml:space="preserve">Udløbet</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nej</t>
+          <t xml:space="preserve">Ja</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026820</t>
+          <t xml:space="preserve">706864, 100063647</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1090,26 +1090,26 @@
         </is>
       </c>
       <c r="F22">
-        <v>3792</v>
+        <v>452</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t xml:space="preserve">311223802</t>
+          <t xml:space="preserve">311122307</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-01-21</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gyldigt</t>
+          <t xml:space="preserve">Udløbet</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nej</t>
+          <t xml:space="preserve">Ja</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">100030239</t>
+          <t xml:space="preserve">100025640</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1140,26 +1140,26 @@
         </is>
       </c>
       <c r="F23">
-        <v>408</v>
+        <v>1440</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve">311223800</t>
+          <t xml:space="preserve">311161386</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-01-21</t>
+          <t xml:space="preserve">2026-02-28</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gyldigt</t>
+          <t xml:space="preserve">Udløbet</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nej</t>
+          <t xml:space="preserve">Ja</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">100047575</t>
+          <t xml:space="preserve">100025821</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1190,16 +1190,16 @@
         </is>
       </c>
       <c r="F24">
-        <v>297</v>
+        <v>996</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">311225730</t>
+          <t xml:space="preserve">311217955</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-01-31</t>
+          <t xml:space="preserve">2026-12-15</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025599</t>
+          <t xml:space="preserve">100030255</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1240,16 +1240,16 @@
         </is>
       </c>
       <c r="F25">
-        <v>255</v>
+        <v>413</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">311226749</t>
+          <t xml:space="preserve">311218022</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-06</t>
+          <t xml:space="preserve">2026-12-15</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025624</t>
+          <t xml:space="preserve">100026820</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1290,16 +1290,16 @@
         </is>
       </c>
       <c r="F26">
-        <v>440</v>
+        <v>3792</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve">311226748</t>
+          <t xml:space="preserve">311223802</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-06</t>
+          <t xml:space="preserve">2027-01-21</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1326,12 +1326,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">190</t>
+          <t xml:space="preserve">147</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">2137707</t>
+          <t xml:space="preserve">100030239</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1340,16 +1340,16 @@
         </is>
       </c>
       <c r="F27">
-        <v>295</v>
+        <v>408</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">311227340</t>
+          <t xml:space="preserve">311223800</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-08</t>
+          <t xml:space="preserve">2027-01-21</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1376,12 +1376,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">230</t>
+          <t xml:space="preserve">147</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">8312706</t>
+          <t xml:space="preserve">100047575</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1390,16 +1390,16 @@
         </is>
       </c>
       <c r="F28">
-        <v>1322</v>
+        <v>297</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">311231330</t>
+          <t xml:space="preserve">311225730</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-08</t>
+          <t xml:space="preserve">2027-01-31</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025655</t>
+          <t xml:space="preserve">100025599</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1440,16 +1440,16 @@
         </is>
       </c>
       <c r="F29">
-        <v>340</v>
+        <v>255</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t xml:space="preserve">311227832</t>
+          <t xml:space="preserve">311226749</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-10</t>
+          <t xml:space="preserve">2027-02-06</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026669</t>
+          <t xml:space="preserve">100025624</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1490,16 +1490,16 @@
         </is>
       </c>
       <c r="F30">
-        <v>626</v>
+        <v>440</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t xml:space="preserve">311227831</t>
+          <t xml:space="preserve">311226748</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-10</t>
+          <t xml:space="preserve">2027-02-06</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1526,12 +1526,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">147</t>
+          <t xml:space="preserve">190</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025685</t>
+          <t xml:space="preserve">2137707</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1540,16 +1540,16 @@
         </is>
       </c>
       <c r="F31">
-        <v>953</v>
+        <v>295</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t xml:space="preserve">311229051</t>
+          <t xml:space="preserve">311227340</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-17</t>
+          <t xml:space="preserve">2027-02-08</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1576,12 +1576,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">147</t>
+          <t xml:space="preserve">230</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028929</t>
+          <t xml:space="preserve">8312706</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="F32">
-        <v>805</v>
+        <v>1322</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">311229048</t>
+          <t xml:space="preserve">311231330</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-17</t>
+          <t xml:space="preserve">2027-02-08</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026522</t>
+          <t xml:space="preserve">100025655</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="F33">
-        <v>300</v>
+        <v>340</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">311230618</t>
+          <t xml:space="preserve">311227832</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-24</t>
+          <t xml:space="preserve">2027-02-10</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1681,25 +1681,25 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026522</t>
+          <t xml:space="preserve">100026669</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F34">
-        <v>376</v>
+        <v>626</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">311230618</t>
+          <t xml:space="preserve">311227831</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-24</t>
+          <t xml:space="preserve">2027-02-10</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026917</t>
+          <t xml:space="preserve">100025685</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1740,16 +1740,16 @@
         </is>
       </c>
       <c r="F35">
-        <v>433</v>
+        <v>953</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">311230540</t>
+          <t xml:space="preserve">311229051</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-24</t>
+          <t xml:space="preserve">2027-02-17</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027090</t>
+          <t xml:space="preserve">100028929</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1790,16 +1790,16 @@
         </is>
       </c>
       <c r="F36">
-        <v>589</v>
+        <v>805</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">311230550</t>
+          <t xml:space="preserve">311229048</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-24</t>
+          <t xml:space="preserve">2027-02-17</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -1831,20 +1831,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029329</t>
+          <t xml:space="preserve">100026522</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F37">
-        <v>1152</v>
+        <v>300</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">311230598</t>
+          <t xml:space="preserve">311230618</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1881,20 +1881,20 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029714</t>
+          <t xml:space="preserve">100026522</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F38">
-        <v>342</v>
+        <v>376</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">311230609</t>
+          <t xml:space="preserve">311230618</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029720</t>
+          <t xml:space="preserve">100026917</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1940,11 +1940,11 @@
         </is>
       </c>
       <c r="F39">
-        <v>1334</v>
+        <v>433</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">311230619</t>
+          <t xml:space="preserve">311230540</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028120</t>
+          <t xml:space="preserve">100027090</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1990,16 +1990,16 @@
         </is>
       </c>
       <c r="F40">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">311230652</t>
+          <t xml:space="preserve">311230550</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-25</t>
+          <t xml:space="preserve">2027-02-24</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2031,25 +2031,25 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">191034</t>
+          <t xml:space="preserve">100029329</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F41">
-        <v>1225</v>
+        <v>1152</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">311230651</t>
+          <t xml:space="preserve">311230598</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-25</t>
+          <t xml:space="preserve">2027-02-24</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028743</t>
+          <t xml:space="preserve">100029714</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2090,16 +2090,16 @@
         </is>
       </c>
       <c r="F42">
-        <v>388</v>
+        <v>342</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">311231234</t>
+          <t xml:space="preserve">311230609</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-28</t>
+          <t xml:space="preserve">2027-02-24</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029487</t>
+          <t xml:space="preserve">100029720</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2140,16 +2140,16 @@
         </is>
       </c>
       <c r="F43">
-        <v>1071</v>
+        <v>1334</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">311231229</t>
+          <t xml:space="preserve">311230619</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-28</t>
+          <t xml:space="preserve">2027-02-24</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2176,12 +2176,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">306</t>
+          <t xml:space="preserve">147</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">5347084</t>
+          <t xml:space="preserve">100028120</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2190,16 +2190,16 @@
         </is>
       </c>
       <c r="F44">
-        <v>1209</v>
+        <v>580</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve">311231683</t>
+          <t xml:space="preserve">311230652</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-02</t>
+          <t xml:space="preserve">2027-02-25</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2231,25 +2231,25 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026820</t>
+          <t xml:space="preserve">100028743</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F45">
-        <v>422</v>
+        <v>388</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">311233222</t>
+          <t xml:space="preserve">311231234</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-09</t>
+          <t xml:space="preserve">2027-02-28</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2281,25 +2281,25 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029530</t>
+          <t xml:space="preserve">100029487</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F46">
-        <v>476</v>
+        <v>1071</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">311233769</t>
+          <t xml:space="preserve">311231229</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-13</t>
+          <t xml:space="preserve">2027-02-28</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">2428914</t>
+          <t xml:space="preserve">5347084</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2340,16 +2340,16 @@
         </is>
       </c>
       <c r="F47">
-        <v>398</v>
+        <v>1209</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t xml:space="preserve">311233782</t>
+          <t xml:space="preserve">311231683</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-13</t>
+          <t xml:space="preserve">2027-03-02</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2381,25 +2381,25 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027252</t>
+          <t xml:space="preserve">100026820</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F48">
-        <v>1486</v>
+        <v>422</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t xml:space="preserve">311234441</t>
+          <t xml:space="preserve">311233222</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-15</t>
+          <t xml:space="preserve">2027-03-09</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2431,25 +2431,25 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025702</t>
+          <t xml:space="preserve">100029530</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F49">
-        <v>29942</v>
+        <v>476</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t xml:space="preserve">311234962</t>
+          <t xml:space="preserve">311233769</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-17</t>
+          <t xml:space="preserve">2027-03-13</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2476,12 +2476,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">147</t>
+          <t xml:space="preserve">306</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026430</t>
+          <t xml:space="preserve">2428914</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2490,16 +2490,16 @@
         </is>
       </c>
       <c r="F50">
-        <v>446</v>
+        <v>398</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t xml:space="preserve">311235357</t>
+          <t xml:space="preserve">311233782</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-20</t>
+          <t xml:space="preserve">2027-03-13</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029530</t>
+          <t xml:space="preserve">100027252</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2540,16 +2540,16 @@
         </is>
       </c>
       <c r="F51">
-        <v>1915</v>
+        <v>1486</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t xml:space="preserve">311236260</t>
+          <t xml:space="preserve">311234441</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-23</t>
+          <t xml:space="preserve">2027-03-15</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2581,25 +2581,25 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025577</t>
+          <t xml:space="preserve">100025702</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F52">
-        <v>525</v>
+        <v>29942</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t xml:space="preserve">311247695</t>
+          <t xml:space="preserve">311234962</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-05-16</t>
+          <t xml:space="preserve">2027-03-17</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026391</t>
+          <t xml:space="preserve">100026430</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2640,16 +2640,16 @@
         </is>
       </c>
       <c r="F53">
-        <v>1000</v>
+        <v>446</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t xml:space="preserve">311248626</t>
+          <t xml:space="preserve">311235357</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-05-19</t>
+          <t xml:space="preserve">2027-03-20</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028380</t>
+          <t xml:space="preserve">100029530</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2690,16 +2690,16 @@
         </is>
       </c>
       <c r="F54">
-        <v>1699</v>
+        <v>1915</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t xml:space="preserve">311248632</t>
+          <t xml:space="preserve">311236260</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-05-19</t>
+          <t xml:space="preserve">2027-03-23</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2731,25 +2731,25 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026777</t>
+          <t xml:space="preserve">100025577</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F55">
-        <v>454</v>
+        <v>525</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t xml:space="preserve">311248790</t>
+          <t xml:space="preserve">311247695</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-05-21</t>
+          <t xml:space="preserve">2027-05-16</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">100047577</t>
+          <t xml:space="preserve">100026391</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2790,16 +2790,16 @@
         </is>
       </c>
       <c r="F56">
-        <v>2679</v>
+        <v>1000</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t xml:space="preserve">311256544</t>
+          <t xml:space="preserve">311248626</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-06-26</t>
+          <t xml:space="preserve">2027-05-19</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -2831,25 +2831,25 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">100030861, 100227750, 100227751</t>
+          <t xml:space="preserve">100028380</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F57">
-        <v>6331</v>
+        <v>1699</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t xml:space="preserve">311268443</t>
+          <t xml:space="preserve">311248632</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-08-24</t>
+          <t xml:space="preserve">2027-05-19</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -2881,7 +2881,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028065</t>
+          <t xml:space="preserve">100026777</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2890,16 +2890,16 @@
         </is>
       </c>
       <c r="F58">
-        <v>1008</v>
+        <v>454</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t xml:space="preserve">311269303</t>
+          <t xml:space="preserve">311248790</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-08-29</t>
+          <t xml:space="preserve">2027-05-21</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026399</t>
+          <t xml:space="preserve">100047577</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2940,16 +2940,16 @@
         </is>
       </c>
       <c r="F59">
-        <v>825</v>
+        <v>2679</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t xml:space="preserve">311285953</t>
+          <t xml:space="preserve">311256544</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-11-27</t>
+          <t xml:space="preserve">2027-06-26</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -2981,25 +2981,25 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026399</t>
+          <t xml:space="preserve">100030861, 100227750, 100227751</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="F60">
-        <v>439</v>
+        <v>6331</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t xml:space="preserve">311285953</t>
+          <t xml:space="preserve">311268443</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-11-27</t>
+          <t xml:space="preserve">2027-08-24</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3031,25 +3031,25 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026399</t>
+          <t xml:space="preserve">100028065</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F61">
-        <v>464</v>
+        <v>1008</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t xml:space="preserve">311285951</t>
+          <t xml:space="preserve">311269303</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-11-27</t>
+          <t xml:space="preserve">2027-08-29</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3086,11 +3086,11 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F62">
-        <v>371</v>
+        <v>825</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -3131,25 +3131,25 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029781</t>
+          <t xml:space="preserve">100026399</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F63">
-        <v>3880</v>
+        <v>439</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t xml:space="preserve">311293188</t>
+          <t xml:space="preserve">311285953</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t xml:space="preserve">2028-01-17</t>
+          <t xml:space="preserve">2027-11-27</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3181,25 +3181,25 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026188</t>
+          <t xml:space="preserve">100026399</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F64">
-        <v>6682</v>
+        <v>464</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t xml:space="preserve">311373826</t>
+          <t xml:space="preserve">311285951</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t xml:space="preserve">2029-04-30</t>
+          <t xml:space="preserve">2027-11-27</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3231,25 +3231,25 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029711</t>
+          <t xml:space="preserve">100026399</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F65">
-        <v>542</v>
+        <v>371</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t xml:space="preserve">311379737</t>
+          <t xml:space="preserve">311285953</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t xml:space="preserve">2029-05-29</t>
+          <t xml:space="preserve">2027-11-27</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3281,7 +3281,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029712</t>
+          <t xml:space="preserve">100029781</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3290,16 +3290,16 @@
         </is>
       </c>
       <c r="F66">
-        <v>311</v>
+        <v>3880</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t xml:space="preserve">311379735</t>
+          <t xml:space="preserve">311293188</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t xml:space="preserve">2029-05-29</t>
+          <t xml:space="preserve">2028-01-17</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029713</t>
+          <t xml:space="preserve">100026188</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3340,16 +3340,16 @@
         </is>
       </c>
       <c r="F67">
-        <v>386</v>
+        <v>6682</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t xml:space="preserve">311379731</t>
+          <t xml:space="preserve">311373826</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t xml:space="preserve">2029-05-29</t>
+          <t xml:space="preserve">2029-04-30</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3381,20 +3381,20 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029713</t>
+          <t xml:space="preserve">100029711</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F68">
-        <v>443</v>
+        <v>542</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t xml:space="preserve">311379734</t>
+          <t xml:space="preserve">311379737</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028525</t>
+          <t xml:space="preserve">100029712</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3440,16 +3440,16 @@
         </is>
       </c>
       <c r="F69">
-        <v>791</v>
+        <v>311</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t xml:space="preserve">311381894</t>
+          <t xml:space="preserve">311379735</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t xml:space="preserve">2029-06-12</t>
+          <t xml:space="preserve">2029-05-29</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3481,7 +3481,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028103</t>
+          <t xml:space="preserve">100029713</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3490,16 +3490,16 @@
         </is>
       </c>
       <c r="F70">
-        <v>300</v>
+        <v>386</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t xml:space="preserve">311384296</t>
+          <t xml:space="preserve">311379731</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t xml:space="preserve">2029-06-24</t>
+          <t xml:space="preserve">2029-05-29</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3531,25 +3531,25 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029627</t>
+          <t xml:space="preserve">100029713</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t xml:space="preserve">16</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F71">
-        <v>1223</v>
+        <v>443</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t xml:space="preserve">311398345</t>
+          <t xml:space="preserve">311379734</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t xml:space="preserve">2029-09-13</t>
+          <t xml:space="preserve">2029-05-29</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3581,25 +3581,25 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t xml:space="preserve">187004</t>
+          <t xml:space="preserve">100028525</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F72">
-        <v>586</v>
+        <v>791</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t xml:space="preserve">311411203</t>
+          <t xml:space="preserve">311381894</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t xml:space="preserve">2029-11-27</t>
+          <t xml:space="preserve">2029-06-12</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3631,25 +3631,25 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t xml:space="preserve">187004</t>
+          <t xml:space="preserve">100028103</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F73">
-        <v>440</v>
+        <v>300</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t xml:space="preserve">311411203</t>
+          <t xml:space="preserve">311384296</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t xml:space="preserve">2029-11-27</t>
+          <t xml:space="preserve">2029-06-24</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3731,25 +3731,25 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027673</t>
+          <t xml:space="preserve">100030861</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">17</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F75">
-        <v>1142</v>
+        <v>3418</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t xml:space="preserve">311473904</t>
+          <t xml:space="preserve">311506322</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t xml:space="preserve">2030-11-08</t>
+          <t xml:space="preserve">2031-03-24</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3781,7 +3781,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t xml:space="preserve">100030861</t>
+          <t xml:space="preserve">100027259</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3790,16 +3790,16 @@
         </is>
       </c>
       <c r="F76">
-        <v>3418</v>
+        <v>3232</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t xml:space="preserve">311506322</t>
+          <t xml:space="preserve">311510299</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t xml:space="preserve">2031-03-24</t>
+          <t xml:space="preserve">2031-04-07</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -3831,7 +3831,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027259</t>
+          <t xml:space="preserve">100027255</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3840,16 +3840,16 @@
         </is>
       </c>
       <c r="F77">
-        <v>3232</v>
+        <v>651</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t xml:space="preserve">311510299</t>
+          <t xml:space="preserve">311511329</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t xml:space="preserve">2031-04-07</t>
+          <t xml:space="preserve">2031-04-10</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027255</t>
+          <t xml:space="preserve">100029030</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3890,16 +3890,16 @@
         </is>
       </c>
       <c r="F78">
-        <v>651</v>
+        <v>568</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t xml:space="preserve">311511329</t>
+          <t xml:space="preserve">311607220</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t xml:space="preserve">2031-04-10</t>
+          <t xml:space="preserve">2032-06-13</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029030</t>
+          <t xml:space="preserve">100028752</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3940,16 +3940,16 @@
         </is>
       </c>
       <c r="F79">
-        <v>568</v>
+        <v>1016</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t xml:space="preserve">311607220</t>
+          <t xml:space="preserve">311712714</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t xml:space="preserve">2032-06-13</t>
+          <t xml:space="preserve">2033-10-05</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -3981,25 +3981,25 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t xml:space="preserve">174850</t>
+          <t xml:space="preserve">100029329</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F80">
-        <v>7906</v>
+        <v>4298</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t xml:space="preserve">311655735</t>
+          <t xml:space="preserve">311715946</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-01-24</t>
+          <t xml:space="preserve">2033-10-18</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -4031,25 +4031,25 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t xml:space="preserve">174851</t>
+          <t xml:space="preserve">100026659</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F81">
-        <v>426</v>
+        <v>474</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t xml:space="preserve">311655850</t>
+          <t xml:space="preserve">311718502</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-01-24</t>
+          <t xml:space="preserve">2033-10-30</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -4081,25 +4081,25 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028752</t>
+          <t xml:space="preserve">100026659</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F82">
-        <v>1016</v>
+        <v>1407</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t xml:space="preserve">311712714</t>
+          <t xml:space="preserve">311718497</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-10-05</t>
+          <t xml:space="preserve">2033-10-30</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029329</t>
+          <t xml:space="preserve">100029488</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4140,16 +4140,16 @@
         </is>
       </c>
       <c r="F83">
-        <v>4298</v>
+        <v>7262</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t xml:space="preserve">311715946</t>
+          <t xml:space="preserve">311718500</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-10-18</t>
+          <t xml:space="preserve">2033-10-30</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -4181,20 +4181,20 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026659</t>
+          <t xml:space="preserve">100029488</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F84">
-        <v>474</v>
+        <v>360</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t xml:space="preserve">311718502</t>
+          <t xml:space="preserve">311718500</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -4231,20 +4231,20 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026659</t>
+          <t xml:space="preserve">100029488</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F85">
-        <v>1407</v>
+        <v>1679</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t xml:space="preserve">311718497</t>
+          <t xml:space="preserve">311718499</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -4281,25 +4281,25 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029488</t>
+          <t xml:space="preserve">100025651</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F86">
-        <v>1679</v>
+        <v>1434</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t xml:space="preserve">311718499</t>
+          <t xml:space="preserve">311718872</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-10-30</t>
+          <t xml:space="preserve">2033-10-31</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025651</t>
+          <t xml:space="preserve">100027661</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4340,11 +4340,11 @@
         </is>
       </c>
       <c r="F87">
-        <v>1434</v>
+        <v>5014</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t xml:space="preserve">311718872</t>
+          <t xml:space="preserve">311718833</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4386,15 +4386,15 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F88">
-        <v>5014</v>
+        <v>1518</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t xml:space="preserve">311718833</t>
+          <t xml:space="preserve">311718915</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -4431,25 +4431,25 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027661</t>
+          <t xml:space="preserve">100025625</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F89">
-        <v>1518</v>
+        <v>575</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t xml:space="preserve">311718915</t>
+          <t xml:space="preserve">311719924</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-10-31</t>
+          <t xml:space="preserve">2033-11-03</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -4481,20 +4481,20 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025625</t>
+          <t xml:space="preserve">100025652</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F90">
-        <v>575</v>
+        <v>2280</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t xml:space="preserve">311719924</t>
+          <t xml:space="preserve">311719943</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -4536,15 +4536,15 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F91">
-        <v>2280</v>
+        <v>910</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t xml:space="preserve">311719943</t>
+          <t xml:space="preserve">311719927</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -4586,15 +4586,15 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F92">
-        <v>910</v>
+        <v>892</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t xml:space="preserve">311719927</t>
+          <t xml:space="preserve">311719941</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -4636,15 +4636,15 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F93">
-        <v>892</v>
+        <v>1827</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t xml:space="preserve">311719941</t>
+          <t xml:space="preserve">311719948</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -4681,20 +4681,20 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025652</t>
+          <t xml:space="preserve">100025653</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F94">
-        <v>1827</v>
+        <v>298</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t xml:space="preserve">311719948</t>
+          <t xml:space="preserve">311719925</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -4731,7 +4731,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025653</t>
+          <t xml:space="preserve">100025654</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4740,11 +4740,11 @@
         </is>
       </c>
       <c r="F95">
-        <v>298</v>
+        <v>390</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t xml:space="preserve">311719925</t>
+          <t xml:space="preserve">311719926</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -4781,7 +4781,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025654</t>
+          <t xml:space="preserve">100026193</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4790,11 +4790,11 @@
         </is>
       </c>
       <c r="F96">
-        <v>390</v>
+        <v>345</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t xml:space="preserve">311719926</t>
+          <t xml:space="preserve">311719933</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -4831,20 +4831,20 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026193</t>
+          <t xml:space="preserve">100026820</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F97">
-        <v>345</v>
+        <v>2018</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t xml:space="preserve">311719933</t>
+          <t xml:space="preserve">311719910</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -4881,25 +4881,25 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026820</t>
+          <t xml:space="preserve">100025625</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F98">
-        <v>2018</v>
+        <v>1906</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t xml:space="preserve">311719910</t>
+          <t xml:space="preserve">311720841</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-11-03</t>
+          <t xml:space="preserve">2033-11-08</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -4931,7 +4931,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025625</t>
+          <t xml:space="preserve">100026838</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4940,16 +4940,16 @@
         </is>
       </c>
       <c r="F99">
-        <v>1906</v>
+        <v>1898</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t xml:space="preserve">311720841</t>
+          <t xml:space="preserve">311722042</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-11-08</t>
+          <t xml:space="preserve">2033-11-14</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -4981,7 +4981,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026838</t>
+          <t xml:space="preserve">100029709</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -4990,11 +4990,11 @@
         </is>
       </c>
       <c r="F100">
-        <v>1898</v>
+        <v>2652</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t xml:space="preserve">311722042</t>
+          <t xml:space="preserve">311721928</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -5031,25 +5031,25 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029709</t>
+          <t xml:space="preserve">100025833</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F101">
-        <v>2652</v>
+        <v>1381</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t xml:space="preserve">311721928</t>
+          <t xml:space="preserve">311722638</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-11-14</t>
+          <t xml:space="preserve">2033-11-16</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5081,20 +5081,20 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025833</t>
+          <t xml:space="preserve">100027933</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F102">
-        <v>1381</v>
+        <v>809</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t xml:space="preserve">311722638</t>
+          <t xml:space="preserve">311722651</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -5131,25 +5131,25 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027933</t>
+          <t xml:space="preserve">100029110</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F103">
-        <v>809</v>
+        <v>348</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t xml:space="preserve">311722651</t>
+          <t xml:space="preserve">311723090</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-11-16</t>
+          <t xml:space="preserve">2033-11-17</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -5181,20 +5181,20 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029110</t>
+          <t xml:space="preserve">100029476</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F104">
-        <v>348</v>
+        <v>2174</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t xml:space="preserve">311723090</t>
+          <t xml:space="preserve">311723087</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -5231,7 +5231,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029476</t>
+          <t xml:space="preserve">100027660</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5240,16 +5240,16 @@
         </is>
       </c>
       <c r="F105">
-        <v>2174</v>
+        <v>6723</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t xml:space="preserve">311723087</t>
+          <t xml:space="preserve">311723274</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-11-17</t>
+          <t xml:space="preserve">2033-11-19</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -5281,25 +5281,25 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027660</t>
+          <t xml:space="preserve">100026025</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F106">
-        <v>6723</v>
+        <v>941</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t xml:space="preserve">311723274</t>
+          <t xml:space="preserve">311723412</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-11-19</t>
+          <t xml:space="preserve">2033-11-20</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -5331,20 +5331,20 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026025</t>
+          <t xml:space="preserve">100027640</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F107">
-        <v>941</v>
+        <v>2139</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t xml:space="preserve">311723412</t>
+          <t xml:space="preserve">311723408</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027640</t>
+          <t xml:space="preserve">100026025</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5390,16 +5390,16 @@
         </is>
       </c>
       <c r="F108">
-        <v>2139</v>
+        <v>2331</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t xml:space="preserve">311723408</t>
+          <t xml:space="preserve">311723961</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-11-20</t>
+          <t xml:space="preserve">2033-11-21</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -5431,20 +5431,20 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026025</t>
+          <t xml:space="preserve">100027673</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">17</t>
         </is>
       </c>
       <c r="F109">
-        <v>2331</v>
+        <v>1142</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t xml:space="preserve">311723961</t>
+          <t xml:space="preserve">311723677</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -5831,7 +5831,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029627</t>
+          <t xml:space="preserve">100027175</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5840,16 +5840,16 @@
         </is>
       </c>
       <c r="F117">
-        <v>7469</v>
+        <v>5031</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t xml:space="preserve">311726343</t>
+          <t xml:space="preserve">311726475</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-12-01</t>
+          <t xml:space="preserve">2033-12-03</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -5881,25 +5881,25 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029627</t>
+          <t xml:space="preserve">100027175</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F118">
-        <v>1826</v>
+        <v>1283</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t xml:space="preserve">311726342</t>
+          <t xml:space="preserve">311726476</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-12-01</t>
+          <t xml:space="preserve">2033-12-03</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -5931,7 +5931,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027175</t>
+          <t xml:space="preserve">100025833</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5940,16 +5940,16 @@
         </is>
       </c>
       <c r="F119">
-        <v>5031</v>
+        <v>2221</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t xml:space="preserve">311726475</t>
+          <t xml:space="preserve">311726873</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-12-03</t>
+          <t xml:space="preserve">2033-12-05</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -5981,25 +5981,25 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027175</t>
+          <t xml:space="preserve">100026309</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F120">
-        <v>1283</v>
+        <v>10865</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t xml:space="preserve">311726476</t>
+          <t xml:space="preserve">311727265</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-12-03</t>
+          <t xml:space="preserve">2033-12-06</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -6031,7 +6031,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025833</t>
+          <t xml:space="preserve">100030249</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -6040,16 +6040,16 @@
         </is>
       </c>
       <c r="F121">
-        <v>2221</v>
+        <v>5199</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t xml:space="preserve">311726873</t>
+          <t xml:space="preserve">311727254</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-12-05</t>
+          <t xml:space="preserve">2033-12-06</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -6081,7 +6081,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026309</t>
+          <t xml:space="preserve">100029769</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -6090,16 +6090,16 @@
         </is>
       </c>
       <c r="F122">
-        <v>10865</v>
+        <v>1176</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t xml:space="preserve">311727265</t>
+          <t xml:space="preserve">311733387</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-12-06</t>
+          <t xml:space="preserve">2034-01-16</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -6131,7 +6131,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t xml:space="preserve">100030249</t>
+          <t xml:space="preserve">100029806</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -6140,16 +6140,16 @@
         </is>
       </c>
       <c r="F123">
-        <v>5199</v>
+        <v>3370</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t xml:space="preserve">311727254</t>
+          <t xml:space="preserve">311734724</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-12-06</t>
+          <t xml:space="preserve">2034-01-20</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -6181,25 +6181,25 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029769</t>
+          <t xml:space="preserve">100028183</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F124">
-        <v>1176</v>
+        <v>375</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t xml:space="preserve">311733387</t>
+          <t xml:space="preserve">311735114</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-01-16</t>
+          <t xml:space="preserve">2034-01-25</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -6231,25 +6231,25 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t xml:space="preserve">191032, 191033</t>
+          <t xml:space="preserve">100028184</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F125">
-        <v>1248</v>
+        <v>562</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t xml:space="preserve">311733392</t>
+          <t xml:space="preserve">311735174</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-01-16</t>
+          <t xml:space="preserve">2034-01-25</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -6281,7 +6281,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029806</t>
+          <t xml:space="preserve">100029540</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -6290,16 +6290,16 @@
         </is>
       </c>
       <c r="F126">
-        <v>3370</v>
+        <v>6815</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t xml:space="preserve">311734724</t>
+          <t xml:space="preserve">311742695</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-01-20</t>
+          <t xml:space="preserve">2034-02-01</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -6331,7 +6331,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028183</t>
+          <t xml:space="preserve">100029540</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -6340,16 +6340,16 @@
         </is>
       </c>
       <c r="F127">
-        <v>375</v>
+        <v>706</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t xml:space="preserve">311735114</t>
+          <t xml:space="preserve">311742696</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-01-25</t>
+          <t xml:space="preserve">2034-02-01</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -6381,25 +6381,25 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028184</t>
+          <t xml:space="preserve">100029540</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F128">
-        <v>562</v>
+        <v>856</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t xml:space="preserve">311735174</t>
+          <t xml:space="preserve">311742694</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-01-25</t>
+          <t xml:space="preserve">2034-02-01</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029540</t>
+          <t xml:space="preserve">100026096</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -6440,16 +6440,16 @@
         </is>
       </c>
       <c r="F129">
-        <v>6815</v>
+        <v>812</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t xml:space="preserve">311742695</t>
+          <t xml:space="preserve">311736735</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-01</t>
+          <t xml:space="preserve">2034-02-02</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -6481,7 +6481,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029540</t>
+          <t xml:space="preserve">100026096</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -6490,16 +6490,16 @@
         </is>
       </c>
       <c r="F130">
-        <v>706</v>
+        <v>1290</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t xml:space="preserve">311742696</t>
+          <t xml:space="preserve">311736733</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-01</t>
+          <t xml:space="preserve">2034-02-02</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -6531,25 +6531,25 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029540</t>
+          <t xml:space="preserve">100029283</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F131">
-        <v>856</v>
+        <v>2340</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t xml:space="preserve">311742694</t>
+          <t xml:space="preserve">311736719</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-01</t>
+          <t xml:space="preserve">2034-02-02</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -6581,7 +6581,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026096</t>
+          <t xml:space="preserve">100029324</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -6590,11 +6590,11 @@
         </is>
       </c>
       <c r="F132">
-        <v>812</v>
+        <v>2412</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t xml:space="preserve">311736735</t>
+          <t xml:space="preserve">311736741</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -6631,25 +6631,25 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026096</t>
+          <t xml:space="preserve">100029349</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F133">
-        <v>1290</v>
+        <v>2532</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t xml:space="preserve">311736733</t>
+          <t xml:space="preserve">311737441</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-02</t>
+          <t xml:space="preserve">2034-02-06</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -6681,7 +6681,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029283</t>
+          <t xml:space="preserve">100029627</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -6690,16 +6690,16 @@
         </is>
       </c>
       <c r="F134">
-        <v>2340</v>
+        <v>7469</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t xml:space="preserve">311736719</t>
+          <t xml:space="preserve">311737458</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-02</t>
+          <t xml:space="preserve">2034-02-06</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -6731,25 +6731,25 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029324</t>
+          <t xml:space="preserve">100029627</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">16</t>
         </is>
       </c>
       <c r="F135">
-        <v>2412</v>
+        <v>1223</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t xml:space="preserve">311736741</t>
+          <t xml:space="preserve">311737458</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-02</t>
+          <t xml:space="preserve">2034-02-06</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -6781,20 +6781,20 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029349</t>
+          <t xml:space="preserve">100029627</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">19</t>
         </is>
       </c>
       <c r="F136">
-        <v>2532</v>
+        <v>912</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t xml:space="preserve">311737441</t>
+          <t xml:space="preserve">311737458</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -6831,25 +6831,25 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025833</t>
+          <t xml:space="preserve">100029627</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F137">
-        <v>467</v>
+        <v>1826</v>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t xml:space="preserve">311738410</t>
+          <t xml:space="preserve">311737458</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-12</t>
+          <t xml:space="preserve">2034-02-06</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -6881,20 +6881,20 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029110</t>
+          <t xml:space="preserve">100025833</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="F138">
-        <v>382</v>
+        <v>467</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t xml:space="preserve">311738404</t>
+          <t xml:space="preserve">311738410</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -6936,15 +6936,15 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="F139">
-        <v>759</v>
+        <v>382</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t xml:space="preserve">311738403</t>
+          <t xml:space="preserve">311738404</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -6981,25 +6981,25 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025884</t>
+          <t xml:space="preserve">100029110</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F140">
-        <v>654</v>
+        <v>759</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t xml:space="preserve">311738624</t>
+          <t xml:space="preserve">311738403</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-13</t>
+          <t xml:space="preserve">2034-02-12</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -7031,25 +7031,25 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025833</t>
+          <t xml:space="preserve">100025884</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F141">
-        <v>1086</v>
+        <v>654</v>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t xml:space="preserve">311738883</t>
+          <t xml:space="preserve">311738624</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-14</t>
+          <t xml:space="preserve">2034-02-13</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -7081,25 +7081,25 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025875</t>
+          <t xml:space="preserve">100025833</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F142">
-        <v>541</v>
+        <v>1086</v>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t xml:space="preserve">311739362</t>
+          <t xml:space="preserve">311738883</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-16</t>
+          <t xml:space="preserve">2034-02-14</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029459</t>
+          <t xml:space="preserve">100025875</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -7140,11 +7140,11 @@
         </is>
       </c>
       <c r="F143">
-        <v>1009</v>
+        <v>541</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t xml:space="preserve">311739367</t>
+          <t xml:space="preserve">311739362</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -7181,7 +7181,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029465</t>
+          <t xml:space="preserve">100029459</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -7190,11 +7190,11 @@
         </is>
       </c>
       <c r="F144">
-        <v>458</v>
+        <v>1009</v>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t xml:space="preserve">311740954</t>
+          <t xml:space="preserve">311739367</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -7236,15 +7236,15 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F145">
-        <v>4137</v>
+        <v>458</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t xml:space="preserve">311739450</t>
+          <t xml:space="preserve">311740954</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -7281,25 +7281,25 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027037</t>
+          <t xml:space="preserve">100029465</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F146">
-        <v>846</v>
+        <v>4137</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t xml:space="preserve">311739928</t>
+          <t xml:space="preserve">311739450</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-20</t>
+          <t xml:space="preserve">2034-02-16</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -7331,25 +7331,25 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028752</t>
+          <t xml:space="preserve">100027037</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F147">
-        <v>594</v>
+        <v>846</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t xml:space="preserve">311740966</t>
+          <t xml:space="preserve">311739928</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-26</t>
+          <t xml:space="preserve">2034-02-20</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -7381,25 +7381,25 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026419</t>
+          <t xml:space="preserve">100028752</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="F148">
-        <v>1965</v>
+        <v>594</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t xml:space="preserve">311741888</t>
+          <t xml:space="preserve">311740966</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-28</t>
+          <t xml:space="preserve">2034-02-26</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -7431,20 +7431,20 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027101</t>
+          <t xml:space="preserve">100026419</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F149">
-        <v>1287</v>
+        <v>1965</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t xml:space="preserve">311741757</t>
+          <t xml:space="preserve">311741888</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
@@ -7481,7 +7481,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027314</t>
+          <t xml:space="preserve">100027101</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -7490,11 +7490,11 @@
         </is>
       </c>
       <c r="F150">
-        <v>1134</v>
+        <v>1287</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t xml:space="preserve">311741762</t>
+          <t xml:space="preserve">311741757</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -7531,7 +7531,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029707</t>
+          <t xml:space="preserve">100027314</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -7540,16 +7540,16 @@
         </is>
       </c>
       <c r="F151">
-        <v>1491</v>
+        <v>1134</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t xml:space="preserve">311742340</t>
+          <t xml:space="preserve">311741762</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-03-01</t>
+          <t xml:space="preserve">2034-02-28</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029708</t>
+          <t xml:space="preserve">100029707</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -7590,11 +7590,11 @@
         </is>
       </c>
       <c r="F152">
-        <v>291</v>
+        <v>1491</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t xml:space="preserve">311742345</t>
+          <t xml:space="preserve">311742340</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -7631,7 +7631,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029822</t>
+          <t xml:space="preserve">100029708</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -7640,11 +7640,11 @@
         </is>
       </c>
       <c r="F153">
-        <v>9353</v>
+        <v>291</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t xml:space="preserve">311743570</t>
+          <t xml:space="preserve">311742345</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
@@ -7681,7 +7681,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026985</t>
+          <t xml:space="preserve">100029822</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -7690,16 +7690,16 @@
         </is>
       </c>
       <c r="F154">
-        <v>814</v>
+        <v>9353</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t xml:space="preserve">311743940</t>
+          <t xml:space="preserve">311743570</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-03-08</t>
+          <t xml:space="preserve">2034-03-01</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -7731,7 +7731,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029646</t>
+          <t xml:space="preserve">100026985</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -7740,11 +7740,11 @@
         </is>
       </c>
       <c r="F155">
-        <v>5305</v>
+        <v>814</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t xml:space="preserve">311743895</t>
+          <t xml:space="preserve">311743940</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -7781,7 +7781,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029790</t>
+          <t xml:space="preserve">100029646</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -7790,16 +7790,16 @@
         </is>
       </c>
       <c r="F156">
-        <v>2615</v>
+        <v>5305</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t xml:space="preserve">311744608</t>
+          <t xml:space="preserve">311743895</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-03-12</t>
+          <t xml:space="preserve">2034-03-08</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -7831,7 +7831,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029802</t>
+          <t xml:space="preserve">100029790</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -7840,11 +7840,11 @@
         </is>
       </c>
       <c r="F157">
-        <v>3280</v>
+        <v>2615</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t xml:space="preserve">311744599</t>
+          <t xml:space="preserve">311744608</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -7881,7 +7881,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029803</t>
+          <t xml:space="preserve">100029802</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -7890,11 +7890,11 @@
         </is>
       </c>
       <c r="F158">
-        <v>3250</v>
+        <v>3280</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t xml:space="preserve">311744589</t>
+          <t xml:space="preserve">311744599</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
@@ -7931,7 +7931,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029307</t>
+          <t xml:space="preserve">100029803</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -7940,16 +7940,16 @@
         </is>
       </c>
       <c r="F159">
-        <v>3120</v>
+        <v>3250</v>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t xml:space="preserve">311767998</t>
+          <t xml:space="preserve">311744589</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-03-14</t>
+          <t xml:space="preserve">2034-03-12</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -7986,15 +7986,15 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F160">
-        <v>2505</v>
+        <v>3120</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t xml:space="preserve">311745373</t>
+          <t xml:space="preserve">311767998</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -8031,20 +8031,20 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029824</t>
+          <t xml:space="preserve">100029307</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F161">
-        <v>4407</v>
+        <v>2505</v>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t xml:space="preserve">311745450</t>
+          <t xml:space="preserve">311745373</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
@@ -8076,12 +8076,12 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t xml:space="preserve">201</t>
+          <t xml:space="preserve">147</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t xml:space="preserve">2252337</t>
+          <t xml:space="preserve">100029824</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
@@ -8090,11 +8090,11 @@
         </is>
       </c>
       <c r="F162">
-        <v>534</v>
+        <v>4407</v>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t xml:space="preserve">311745449</t>
+          <t xml:space="preserve">311745450</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -8126,12 +8126,12 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t xml:space="preserve">147</t>
+          <t xml:space="preserve">201</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029472</t>
+          <t xml:space="preserve">2252337</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -8140,16 +8140,16 @@
         </is>
       </c>
       <c r="F163">
-        <v>4687</v>
+        <v>534</v>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t xml:space="preserve">311746471</t>
+          <t xml:space="preserve">311745449</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-03-19</t>
+          <t xml:space="preserve">2034-03-14</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t xml:space="preserve">174465, 174466, 174468, 174469</t>
+          <t xml:space="preserve">100029472</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -8190,16 +8190,16 @@
         </is>
       </c>
       <c r="F164">
-        <v>13136</v>
+        <v>4687</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t xml:space="preserve">311746996</t>
+          <t xml:space="preserve">311746471</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-03-21</t>
+          <t xml:space="preserve">2034-03-19</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">

</xml_diff>